<commit_message>
feat: place recovered SMD footprints and record draft assembly positions
</commit_message>
<xml_diff>
--- a/fancontroller_BOM_populated.xlsx
+++ b/fancontroller_BOM_populated.xlsx
@@ -10,10 +10,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PCB Assembly" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Off-board options" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Placement draft" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PCB Assembly'!$A$1:$K$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Off-board options'!$A$1:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Placement draft'!$A$1:$G$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +23,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="9">
     <font>
       <name val="Calibri"/>
@@ -72,7 +76,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -99,6 +103,16 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00183153"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F5FA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -112,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -149,6 +163,18 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1581,4 +1607,546 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="75" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>X on KiCad board (mm)</t>
+        </is>
+      </c>
+      <c r="C1" s="14" t="inlineStr">
+        <is>
+          <t>Y on KiCad board (mm)</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>Rotation (deg)</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>Max pad-center offset from supplied F.Paste (mm)</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="G1" s="14" t="inlineStr">
+        <is>
+          <t>Review status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="n">
+        <v>81.28</v>
+      </c>
+      <c r="C2" s="16" t="n">
+        <v>160.909</v>
+      </c>
+      <c r="D2" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="16" t="n">
+        <v>0.0125</v>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>F.Paste Gerber</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>Placed; exact value and body size to confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="n">
+        <v>94.996</v>
+      </c>
+      <c r="C3" s="17" t="n">
+        <v>155.448</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E3" s="17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>F.Paste Gerber</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>Placed; library pad centers differ from paste</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="n">
+        <v>94.996</v>
+      </c>
+      <c r="C4" s="16" t="n">
+        <v>164.592</v>
+      </c>
+      <c r="D4" s="15" t="n">
+        <v>90</v>
+      </c>
+      <c r="E4" s="16" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>F.Paste Gerber</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>Placed; library pad centers differ from paste</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="n">
+        <v>96.52</v>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>172.4295</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>F.Paste Gerber</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Placed; value and body size to confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>84.328</v>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>147.574</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>135</v>
+      </c>
+      <c r="E6" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>F.Paste Gerber</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>Placed; polarity and can size must be verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>IC1</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="n">
+        <v>95.8596</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>150.5204</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>F.Paste Gerber</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Placed; SOIC row spacing differs from paste</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>IC2</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="n">
+        <v>90.17</v>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>158.496</v>
+      </c>
+      <c r="D8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="16" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>F.Paste Gerber</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>Placed; SOIC row spacing differs from paste</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>IC3</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="n">
+        <v>90.17</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>167.64</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>F.Paste Gerber</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>Placed; SOIC row spacing differs from paste</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>REG1</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>89.6366</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>143.4338</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <v>-45</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>0.2251</v>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>F.Paste Gerber</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>Placed; SOIC row spacing and pin orientation to verify</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="n">
+        <v>81.28</v>
+      </c>
+      <c r="C11" s="17" t="n">
+        <v>154.432</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>F.Paste Gerber</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>Placed</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="n">
+        <v>81.28</v>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>157.48</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>F.Paste Gerber</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>Placed</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="n">
+        <v>81.28</v>
+      </c>
+      <c r="C13" s="17" t="n">
+        <v>164.465</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>F.Paste Gerber</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>Placed</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="n">
+        <v>81.28</v>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>167.513</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="16" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>F.Paste Gerber</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>Placed</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="n">
+        <v>90.3335</v>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>162.56</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>F.Paste Gerber</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>Placed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="n">
+        <v>90.17</v>
+      </c>
+      <c r="C16" s="16" t="n">
+        <v>172.72</v>
+      </c>
+      <c r="D16" s="15" t="n"/>
+      <c r="E16" s="16" t="n"/>
+      <c r="F16" s="15" t="inlineStr">
+        <is>
+          <t>PTH drill and board image</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>Pending; three 2.54 mm drill holes, board interface needs footprint selection</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>J1</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="n">
+        <v>99.568</v>
+      </c>
+      <c r="C17" s="17" t="n">
+        <v>163.322</v>
+      </c>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="17" t="n"/>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>PTH drill and board image</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>Pending; four 2.54 mm drill holes, Molex footprint needs confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>J2</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="n">
+        <v>100.076</v>
+      </c>
+      <c r="C18" s="16" t="n">
+        <v>155.956</v>
+      </c>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="16" t="n"/>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>PTH drill and board image</t>
+        </is>
+      </c>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>Pending; inferred two-pin power connector needs part selection</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G18"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: obtain five-board SMT quote with stocked 12 V replacements
</commit_message>
<xml_diff>
--- a/fancontroller_BOM_populated.xlsx
+++ b/fancontroller_BOM_populated.xlsx
@@ -646,22 +646,22 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>TS2938CS50 RLG</t>
+          <t>KF50BD-TR</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Taiwan Semiconductor</t>
+          <t>STMicroelectronics</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Package_SO:SOIC-8_3.9x4.9mm_P1.27mm</t>
+          <t>Recovered2018:SOIC-8_3.9x4.9mm_P1.27mm</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>C557546</t>
+          <t>C222151</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -671,17 +671,17 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Candidate; verify stock</t>
+          <t>Stocked quote replacement; 12 V only</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Original BOM says TS2938CS50; RLG is the catalog order variant. Regulator is not yet placed in schematic.</t>
+          <t>Same pinout and active-low inhibit. 500 mA; input limit 20 V. Original 12-28 V silk is not valid for this build.</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C557546.html</t>
+          <t>https://www.st.com/resource/en/datasheet/kfxx.pdf</t>
         </is>
       </c>
     </row>
@@ -701,22 +701,22 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>C1206C561K5RAC7800</t>
+          <t>CC1206JRNPO9BN561</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>KEMET</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_1206_3216Metric</t>
+          <t>Recovered2018:C_1206_3216Metric_Pad1.42x1.75mm_HandSolder</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>C2178336</t>
+          <t>C577166</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -726,17 +726,17 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Exact MPN; out of stock</t>
+          <t>Stocked quote replacement</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>LCSC listing showed zero stock at research time; choose an approved substitute before assembly.</t>
+          <t>560 pF, 50 V, NP0, 5%, 1206. Replaces original 10% X7R timing capacitor.</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-image/C2178336.html</t>
+          <t>https://jlcpcb.com/partdetail/YAGEO-CC1206JRNPO9BN561/C577166</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_0603_1608Metric</t>
+          <t>Recovered2018:C_0603_1608Metric_Pad1.05x0.95mm_HandSolder</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -811,22 +811,22 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>C1206C101KCRACTU</t>
+          <t>CC1206JRNPOBBN101</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>KEMET</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_1206_3216Metric</t>
+          <t>Recovered2018:C_1206_3216Metric_Pad1.42x1.75mm_HandSolder</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>C2178961</t>
+          <t>C113888</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -836,17 +836,17 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Exact MPN; verify stock</t>
+          <t>Stocked quote replacement</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Original BOM suggested this part.</t>
+          <t>100 pF, 500 V, NP0, 5%, 1206. Retains capacitance, voltage rating and package.</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2178961.html</t>
+          <t>https://jlcpcb.com/partdetail/YAGEO-CC1206JRNPOBBN101/C113888</t>
         </is>
       </c>
     </row>
@@ -861,25 +861,29 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>47 µF, 10 V polarized aluminum capacitor</t>
+          <t>47 µF, 35 V polarized aluminum capacitor</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>UUL1A470MCL1GS</t>
+          <t>EEEFK1V470AP</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Nichicon</t>
+          <t>Panasonic</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:CP_Elec_6.3x5.8</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr"/>
+          <t>Recovered2018:CP_Elec_6.3x5.8</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>C336786</t>
+        </is>
+      </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
           <t>SMT</t>
@@ -887,17 +891,17 @@
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>MPN known; footprint review</t>
+          <t>Stocked quote replacement</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>Original BOM says 6.6 × 6.6 mm can; manufacturer table lists 6.3 × 5.8 mm. Verify land pattern and polarity.</t>
+          <t>Same 6.3x5.8 mm case; 0.36 ohm impedance. Rated 2000 h at 105 C versus original 5000 h. Native polarity 315 degrees.</t>
         </is>
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>https://datasheet.lcsc.com/datasheet/pdf/5e881fdd0cb26265cc6618695efc845e.pdf?productCode=C1952683</t>
+          <t>https://industrial.panasonic.com/ww/products/pt/aluminum-cap-smd/models/EEEFK1V470AP</t>
         </is>
       </c>
     </row>
@@ -927,7 +931,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Package_SO:SOIC-8_3.9x4.9mm_P1.27mm</t>
+          <t>Recovered2018:SOIC-8_3.9x4.9mm_P1.27mm</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -982,7 +986,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Package_SO:SOIC-8_3.9x4.9mm_P1.27mm</t>
+          <t>Recovered2018:SOIC-8_3.9x4.9mm_P1.27mm</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -1037,7 +1041,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_1206_3216Metric</t>
+          <t>Recovered2018:R_1206_3216Metric_Pad1.42x1.75mm_HandSolder</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1092,7 +1096,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_1206_3216Metric</t>
+          <t>Recovered2018:R_1206_3216Metric_Pad1.42x1.75mm_HandSolder</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -1147,10 +1151,14 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_1206_3216Metric</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr"/>
+          <t>Recovered2018:R_1206_3216Metric_Pad1.42x1.75mm_HandSolder</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>C163368</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
           <t>SMT</t>
@@ -1158,7 +1166,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>MPN known; LCSC match open</t>
+          <t>Exact MPN matched to JLCPCB</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1166,7 +1174,11 @@
           <t>Original BOM test-circuit part; obtain a current JLC/LCSC listing.</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>https://jlcpcb.com/partdetail/YAGEO-RC1206FR079K1L/C163368</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -1194,7 +1206,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_1206_3216Metric</t>
+          <t>Recovered2018:R_1206_3216Metric_Pad1.42x1.75mm_HandSolder</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -1576,7 +1588,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>KiCad schematic symbols are placed but not wired; regulator is not yet placed. Gerber-derived board has artwork but no component footprints or net assignments.</t>
+          <t>17 schematic symbols remain unwired (ERC 79). Board has 14 SMT footprints matching original paste pads within 0.001 mm, but no nets (DRC 639). Courtyard violations: 0.</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1600,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Do not use this workbook as a release BOM until footprints, schematic connectivity, substitute parts, JLCPCB stock, and assembly method are verified.</t>
+          <t>Quote: five boards, 14 SMT parts each, 12 V supply. Stocked replacements are in PCB Assembly and JLCPCB_Quote/BOM.csv. P1/J1/J2 remain for hand assembly. Electrical validation is incomplete.</t>
         </is>
       </c>
     </row>
@@ -1680,7 +1692,7 @@
         <v>0</v>
       </c>
       <c r="E2" s="16" t="n">
-        <v>0.0125</v>
+        <v>0</v>
       </c>
       <c r="F2" s="15" t="inlineStr">
         <is>
@@ -1689,7 +1701,7 @@
       </c>
       <c r="G2" s="15" t="inlineStr">
         <is>
-          <t>Placed; exact value and body size to confirm</t>
+          <t>Pad centers and pad angles match supplied Gerber (&lt;0.001 mm); quote geometry verified; electrical validation incomplete.</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1721,7 @@
         <v>90</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -1718,7 +1730,7 @@
       </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
-          <t>Placed; library pad centers differ from paste</t>
+          <t>Pad centers and pad angles match supplied Gerber (&lt;0.001 mm); quote geometry verified; electrical validation incomplete.</t>
         </is>
       </c>
     </row>
@@ -1738,7 +1750,7 @@
         <v>90</v>
       </c>
       <c r="E4" s="16" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
@@ -1747,7 +1759,7 @@
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>Placed; library pad centers differ from paste</t>
+          <t>Pad centers and pad angles match supplied Gerber (&lt;0.001 mm); quote geometry verified; electrical validation incomplete.</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1779,7 @@
         <v>90</v>
       </c>
       <c r="E5" s="17" t="n">
-        <v>0.013</v>
+        <v>0.0005000000000165983</v>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
@@ -1776,7 +1788,7 @@
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>Placed; value and body size to confirm</t>
+          <t>Pad centers and pad angles match supplied Gerber (&lt;0.001 mm); quote geometry verified; electrical validation incomplete.</t>
         </is>
       </c>
     </row>
@@ -1793,10 +1805,10 @@
         <v>147.574</v>
       </c>
       <c r="D6" s="15" t="n">
-        <v>135</v>
+        <v>315</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>0</v>
+        <v>4.372800346421952e-07</v>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
@@ -1805,7 +1817,7 @@
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>Placed; polarity and can size must be verified</t>
+          <t>Pad centers and pad angles match supplied Gerber (&lt;0.001 mm); quote geometry verified; electrical validation incomplete.</t>
         </is>
       </c>
     </row>
@@ -1825,7 +1837,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>0.225</v>
+        <v>0.0003999999999848569</v>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
@@ -1834,7 +1846,7 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>Placed; SOIC row spacing differs from paste</t>
+          <t>Pad centers and pad angles match supplied Gerber (&lt;0.001 mm); quote geometry verified; electrical validation incomplete.</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1866,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="16" t="n">
-        <v>0.225</v>
+        <v>2.842170943040401e-14</v>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
@@ -1863,7 +1875,7 @@
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>Placed; SOIC row spacing differs from paste</t>
+          <t>Pad centers and pad angles match supplied Gerber (&lt;0.001 mm); quote geometry verified; electrical validation incomplete.</t>
         </is>
       </c>
     </row>
@@ -1883,7 +1895,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="17" t="n">
-        <v>0.225</v>
+        <v>2.842170943040401e-14</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
@@ -1892,7 +1904,7 @@
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>Placed; SOIC row spacing differs from paste</t>
+          <t>Pad centers and pad angles match supplied Gerber (&lt;0.001 mm); quote geometry verified; electrical validation incomplete.</t>
         </is>
       </c>
     </row>
@@ -1909,10 +1921,10 @@
         <v>143.4338</v>
       </c>
       <c r="D10" s="15" t="n">
-        <v>-45</v>
+        <v>315</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>0.2251</v>
+        <v>0.0002004968828997431</v>
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
@@ -1921,7 +1933,7 @@
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>Placed; SOIC row spacing and pin orientation to verify</t>
+          <t>Pad centers and pad angles match supplied Gerber (&lt;0.001 mm); quote geometry verified; electrical validation incomplete.</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1953,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="17" t="n">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
@@ -1950,7 +1962,7 @@
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>Placed</t>
+          <t>Pad centers and pad angles match supplied Gerber (&lt;0.001 mm); quote geometry verified; electrical validation incomplete.</t>
         </is>
       </c>
     </row>
@@ -1970,7 +1982,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="16" t="n">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
@@ -1979,7 +1991,7 @@
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>Placed</t>
+          <t>Pad centers and pad angles match supplied Gerber (&lt;0.001 mm); quote geometry verified; electrical validation incomplete.</t>
         </is>
       </c>
     </row>
@@ -1999,7 +2011,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="17" t="n">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
@@ -2008,7 +2020,7 @@
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>Placed</t>
+          <t>Pad centers and pad angles match supplied Gerber (&lt;0.001 mm); quote geometry verified; electrical validation incomplete.</t>
         </is>
       </c>
     </row>
@@ -2028,7 +2040,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="F14" s="15" t="inlineStr">
         <is>
@@ -2037,7 +2049,7 @@
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>Placed</t>
+          <t>Pad centers and pad angles match supplied Gerber (&lt;0.001 mm); quote geometry verified; electrical validation incomplete.</t>
         </is>
       </c>
     </row>
@@ -2057,7 +2069,7 @@
         <v>0</v>
       </c>
       <c r="E15" s="17" t="n">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
@@ -2066,7 +2078,7 @@
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>Placed</t>
+          <t>Pad centers and pad angles match supplied Gerber (&lt;0.001 mm); quote geometry verified; electrical validation incomplete.</t>
         </is>
       </c>
     </row>

</xml_diff>